<commit_message>
Validate shared division award counts
</commit_message>
<xml_diff>
--- a/2025-FLL-Qualifier-Tournaments-with-divisions.xlsx
+++ b/2025-FLL-Qualifier-Tournaments-with-divisions.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github-projects\FLL-Season-and-Tournament-Management\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59CA0D2A-E778-4F4F-9208-ECE73D0DAC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B50901C-0287-4708-9BDE-DF397758D069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="3" xr2:uid="{0852510A-0402-494B-87EA-4B91755641F1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{0852510A-0402-494B-87EA-4B91755641F1}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="9" r:id="rId1"/>
@@ -3797,123 +3797,6 @@
         <name val="Calibri"/>
         <family val="2"/>
         <scheme val="none"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
       </font>
     </dxf>
     <dxf>
@@ -4657,6 +4540,123 @@
         <scheme val="none"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -5057,53 +5057,53 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2C2782E-8D00-4650-88D9-CBAFC7F68F2F}" name="Summary" displayName="Summary" ref="A1:U17" totalsRowShown="0" headerRowDxfId="61" dataDxfId="60">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F2C2782E-8D00-4650-88D9-CBAFC7F68F2F}" name="Summary" displayName="Summary" ref="A1:U17" totalsRowShown="0" headerRowDxfId="52" dataDxfId="51">
   <autoFilter ref="A1:U17" xr:uid="{BE3A572B-CA44-4747-B917-FCB04945D86D}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{BF1F7E71-E66D-4B0C-89F9-16ABE7AA3A1D}" name="Item" dataDxfId="59"/>
-    <tableColumn id="2" xr3:uid="{D668F0F3-57FC-4961-897C-AEAADA4362DF}" name="Newport_News" dataDxfId="58"/>
-    <tableColumn id="3" xr3:uid="{0D9B86E2-CF98-40AA-AE69-31D927B8512D}" name="Henrico_Godwin" dataDxfId="57"/>
-    <tableColumn id="4" xr3:uid="{23C8D6E7-CDEC-4B0A-A2FB-20309BE65D99}" name="Glen_Allen" dataDxfId="56"/>
-    <tableColumn id="5" xr3:uid="{7D2B892A-A9F7-4E1F-A90C-EDFB5485B1AE}" name="Martinsville" dataDxfId="55"/>
-    <tableColumn id="6" xr3:uid="{8187554D-A12A-428A-A29B-8D92D08DABAE}" name="Norfolk" dataDxfId="54"/>
-    <tableColumn id="7" xr3:uid="{DD480F0C-B63E-4836-8615-3CBD1B456110}" name="Blacksburg" dataDxfId="53"/>
-    <tableColumn id="8" xr3:uid="{E55B54A1-2E1E-4E81-B861-1254ADE8C3C7}" name="Abingdon" dataDxfId="52"/>
-    <tableColumn id="9" xr3:uid="{F22D09BC-D7FE-45B8-B3AA-4A632D4F0531}" name="Charlottesville" dataDxfId="51"/>
-    <tableColumn id="10" xr3:uid="{7703ECD1-EFAA-4F63-9050-425B0B9A7A45}" name="Manassas_1" dataDxfId="50"/>
-    <tableColumn id="11" xr3:uid="{4286384C-47D1-4C43-897C-4839794136FF}" name="Chantilly" dataDxfId="49"/>
-    <tableColumn id="12" xr3:uid="{B50C72AA-6A79-402B-807E-793A9D5D98BA}" name="Manassas_2" dataDxfId="48"/>
-    <tableColumn id="13" xr3:uid="{60408385-DDF9-45CC-BF1F-54054F87E546}" name="Richmond" dataDxfId="47"/>
-    <tableColumn id="14" xr3:uid="{E7460837-F884-44D7-8EB3-95FB2CE2AC4A}" name="DC-McKinley" dataDxfId="46"/>
-    <tableColumn id="15" xr3:uid="{28672377-5931-492B-B0DB-D60F205A71D1}" name="DC-Friendship" dataDxfId="45"/>
-    <tableColumn id="16" xr3:uid="{DE2FA6CE-1FFD-4892-9A73-81E4AA8ECB84}" name="Ashburn" dataDxfId="44"/>
-    <tableColumn id="17" xr3:uid="{20F96C36-71C3-4737-9B8E-E6966F5E8BD5}" name="Alexandria" dataDxfId="43"/>
-    <tableColumn id="23" xr3:uid="{3DCA30AE-A6A2-4AB3-9296-B49431379BE7}" name="Henrico_Freeman" dataDxfId="42"/>
-    <tableColumn id="24" xr3:uid="{DF427F3F-27AF-4F92-A380-9BA8F66764C4}" name="Hayfield_1" dataDxfId="41"/>
-    <tableColumn id="25" xr3:uid="{8B42BC8B-8E1F-4C9D-BAD3-BE48C8E8FB14}" name="Hayfield_2" dataDxfId="40"/>
-    <tableColumn id="18" xr3:uid="{B503E49C-2072-4A2D-8458-9F5C833A9CE4}" name="Test" dataDxfId="39"/>
+    <tableColumn id="1" xr3:uid="{BF1F7E71-E66D-4B0C-89F9-16ABE7AA3A1D}" name="Item" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{D668F0F3-57FC-4961-897C-AEAADA4362DF}" name="Newport_News" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{0D9B86E2-CF98-40AA-AE69-31D927B8512D}" name="Henrico_Godwin" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{23C8D6E7-CDEC-4B0A-A2FB-20309BE65D99}" name="Glen_Allen" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{7D2B892A-A9F7-4E1F-A90C-EDFB5485B1AE}" name="Martinsville" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{8187554D-A12A-428A-A29B-8D92D08DABAE}" name="Norfolk" dataDxfId="45"/>
+    <tableColumn id="7" xr3:uid="{DD480F0C-B63E-4836-8615-3CBD1B456110}" name="Blacksburg" dataDxfId="44"/>
+    <tableColumn id="8" xr3:uid="{E55B54A1-2E1E-4E81-B861-1254ADE8C3C7}" name="Abingdon" dataDxfId="43"/>
+    <tableColumn id="9" xr3:uid="{F22D09BC-D7FE-45B8-B3AA-4A632D4F0531}" name="Charlottesville" dataDxfId="42"/>
+    <tableColumn id="10" xr3:uid="{7703ECD1-EFAA-4F63-9050-425B0B9A7A45}" name="Manassas_1" dataDxfId="41"/>
+    <tableColumn id="11" xr3:uid="{4286384C-47D1-4C43-897C-4839794136FF}" name="Chantilly" dataDxfId="40"/>
+    <tableColumn id="12" xr3:uid="{B50C72AA-6A79-402B-807E-793A9D5D98BA}" name="Manassas_2" dataDxfId="39"/>
+    <tableColumn id="13" xr3:uid="{60408385-DDF9-45CC-BF1F-54054F87E546}" name="Richmond" dataDxfId="38"/>
+    <tableColumn id="14" xr3:uid="{E7460837-F884-44D7-8EB3-95FB2CE2AC4A}" name="DC-McKinley" dataDxfId="37"/>
+    <tableColumn id="15" xr3:uid="{28672377-5931-492B-B0DB-D60F205A71D1}" name="DC-Friendship" dataDxfId="36"/>
+    <tableColumn id="16" xr3:uid="{DE2FA6CE-1FFD-4892-9A73-81E4AA8ECB84}" name="Ashburn" dataDxfId="35"/>
+    <tableColumn id="17" xr3:uid="{20F96C36-71C3-4737-9B8E-E6966F5E8BD5}" name="Alexandria" dataDxfId="34"/>
+    <tableColumn id="23" xr3:uid="{3DCA30AE-A6A2-4AB3-9296-B49431379BE7}" name="Henrico_Freeman" dataDxfId="33"/>
+    <tableColumn id="24" xr3:uid="{DF427F3F-27AF-4F92-A380-9BA8F66764C4}" name="Hayfield_1" dataDxfId="32"/>
+    <tableColumn id="25" xr3:uid="{8B42BC8B-8E1F-4C9D-BAD3-BE48C8E8FB14}" name="Hayfield_2" dataDxfId="31"/>
+    <tableColumn id="18" xr3:uid="{B503E49C-2072-4A2D-8458-9F5C833A9CE4}" name="Test" dataDxfId="30"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7B16C461-5BC9-4866-8279-89BA5266DF3D}" name="TournamentList" displayName="TournamentList" ref="A1:N2" insertRow="1" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{7B16C461-5BC9-4866-8279-89BA5266DF3D}" name="TournamentList" displayName="TournamentList" ref="A1:N2" insertRow="1" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A1:N2" xr:uid="{7B16C461-5BC9-4866-8279-89BA5266DF3D}"/>
   <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{41ADFF91-8737-40DB-B5BF-F1FE1207C8F3}" name="Short Name" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{8C615F1E-6A8E-4D42-B4AF-FF0093E0EF5D}" name="Long Name" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{60E0111B-D905-482F-A1BA-7C258739C404}" name="Date" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{CD391DEA-3CAA-4B07-95CE-E82E2C75503C}" name="OJS_FileName" dataDxfId="33"/>
-    <tableColumn id="16" xr3:uid="{589BE392-D192-48FB-BD40-5702D58DF938}" name="J_AWD_CHAMP" dataDxfId="32"/>
-    <tableColumn id="17" xr3:uid="{FA8383F9-491B-4BD1-9FCC-9EAEE62C41B4}" name="J_AWD_IP" dataDxfId="31"/>
-    <tableColumn id="18" xr3:uid="{88F56DA0-0566-4649-B005-071E67DC4D86}" name="J_AWD_RD" dataDxfId="30"/>
-    <tableColumn id="19" xr3:uid="{931DAD6B-FFB1-4AF8-BE54-1AC7E9E2A345}" name="J_AWD_CV" dataDxfId="29"/>
-    <tableColumn id="20" xr3:uid="{D867B27A-ED2F-4865-98DB-CECEFC2403A4}" name="J_AWD_Judges" dataDxfId="28"/>
-    <tableColumn id="21" xr3:uid="{10865F36-DA77-4444-9FB1-1A3A1ED5430D}" name="P_AWD_RG" dataDxfId="27"/>
-    <tableColumn id="22" xr3:uid="{7425636E-CB8A-4393-9F08-52250AF37B31}" name="J_AWD_BT" dataDxfId="26"/>
-    <tableColumn id="23" xr3:uid="{0D14A66D-182C-4868-A20E-357F8EC3C9C7}" name="J_AWD_RisAll" dataDxfId="25"/>
-    <tableColumn id="24" xr3:uid="{635C8BEE-8813-4870-B73F-F5B068653F7E}" name="J_AWD_CL" dataDxfId="24"/>
-    <tableColumn id="6" xr3:uid="{D992314A-D45D-4770-AE5E-BCF9A32099CC}" name="ADV" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{41ADFF91-8737-40DB-B5BF-F1FE1207C8F3}" name="Short Name" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{8C615F1E-6A8E-4D42-B4AF-FF0093E0EF5D}" name="Long Name" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{60E0111B-D905-482F-A1BA-7C258739C404}" name="Date" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{CD391DEA-3CAA-4B07-95CE-E82E2C75503C}" name="OJS_FileName" dataDxfId="24"/>
+    <tableColumn id="16" xr3:uid="{589BE392-D192-48FB-BD40-5702D58DF938}" name="J_AWD_CHAMP" dataDxfId="23"/>
+    <tableColumn id="17" xr3:uid="{FA8383F9-491B-4BD1-9FCC-9EAEE62C41B4}" name="J_AWD_IP" dataDxfId="22"/>
+    <tableColumn id="18" xr3:uid="{88F56DA0-0566-4649-B005-071E67DC4D86}" name="J_AWD_RD" dataDxfId="21"/>
+    <tableColumn id="19" xr3:uid="{931DAD6B-FFB1-4AF8-BE54-1AC7E9E2A345}" name="J_AWD_CV" dataDxfId="20"/>
+    <tableColumn id="20" xr3:uid="{D867B27A-ED2F-4865-98DB-CECEFC2403A4}" name="J_AWD_Judges" dataDxfId="19"/>
+    <tableColumn id="21" xr3:uid="{10865F36-DA77-4444-9FB1-1A3A1ED5430D}" name="P_AWD_RG" dataDxfId="18"/>
+    <tableColumn id="22" xr3:uid="{7425636E-CB8A-4393-9F08-52250AF37B31}" name="J_AWD_BT" dataDxfId="17"/>
+    <tableColumn id="23" xr3:uid="{0D14A66D-182C-4868-A20E-357F8EC3C9C7}" name="J_AWD_RisAll" dataDxfId="16"/>
+    <tableColumn id="24" xr3:uid="{635C8BEE-8813-4870-B73F-F5B068653F7E}" name="J_AWD_CL" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{D992314A-D45D-4770-AE5E-BCF9A32099CC}" name="ADV" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5114,42 +5114,42 @@
   <autoFilter ref="A1:M38" xr:uid="{B6A06E95-68C8-4940-B680-2C0995F031C3}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{13A1917A-5FA7-45FA-916C-27FE0F8E0A97}" name="Short Name"/>
-    <tableColumn id="7" xr3:uid="{9239BE62-20DE-4C00-B4EA-0F023772BA66}" name="Long Name" dataDxfId="22"/>
-    <tableColumn id="8" xr3:uid="{3D68214D-736A-4612-8FC4-63A9FB374D80}" name="Date" dataDxfId="21"/>
+    <tableColumn id="7" xr3:uid="{9239BE62-20DE-4C00-B4EA-0F023772BA66}" name="Long Name" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{3D68214D-736A-4612-8FC4-63A9FB374D80}" name="Date" dataDxfId="12"/>
     <tableColumn id="41" xr3:uid="{FD3155A7-7337-4CCF-8C34-CE92DA3A68FB}" name="Div"/>
-    <tableColumn id="2" xr3:uid="{6D5A88F8-4F5F-4888-9747-1A76C77056E2}" name="Helper" dataDxfId="20">
+    <tableColumn id="2" xr3:uid="{6D5A88F8-4F5F-4888-9747-1A76C77056E2}" name="Helper" dataDxfId="11">
       <calculatedColumnFormula>DivTournamentList[[#This Row],[Short Name]]&amp;DivTournamentList[[#This Row],[Div]]</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="6" xr3:uid="{A8A35723-08A9-4CA4-B0A0-9D1F1126A77A}" name="OJS_FileName">
       <calculatedColumnFormula>"2025-vadc-fll-challenge-Unearthed-ojs-" &amp; DivTournamentList[[#This Row],[Helper]] &amp; ".xlsm"</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{77D06F86-14CD-457E-96E9-6EB6B7AFEB60}" name="J_AWD_CHAMP" dataDxfId="19"/>
-    <tableColumn id="22" xr3:uid="{996BB723-6D12-4C0A-9F23-3D5E78572496}" name="J_AWD_RD" dataDxfId="18"/>
-    <tableColumn id="23" xr3:uid="{3C6ED932-F80C-4988-A3E5-3724D007931F}" name="J_AWD_IP" dataDxfId="17"/>
-    <tableColumn id="24" xr3:uid="{C65C332E-AD2E-45F0-90A7-77C4F6D09E4D}" name="J_AWD_CV" dataDxfId="16"/>
-    <tableColumn id="25" xr3:uid="{CC3139B7-4C8A-4742-964E-81B4CC04BA42}" name="P_AWD_RG" dataDxfId="15"/>
+    <tableColumn id="21" xr3:uid="{77D06F86-14CD-457E-96E9-6EB6B7AFEB60}" name="J_AWD_CHAMP" dataDxfId="10"/>
+    <tableColumn id="22" xr3:uid="{996BB723-6D12-4C0A-9F23-3D5E78572496}" name="J_AWD_RD" dataDxfId="9"/>
+    <tableColumn id="23" xr3:uid="{3C6ED932-F80C-4988-A3E5-3724D007931F}" name="J_AWD_IP" dataDxfId="8"/>
+    <tableColumn id="24" xr3:uid="{C65C332E-AD2E-45F0-90A7-77C4F6D09E4D}" name="J_AWD_CV" dataDxfId="7"/>
+    <tableColumn id="25" xr3:uid="{CC3139B7-4C8A-4742-964E-81B4CC04BA42}" name="P_AWD_RG" dataDxfId="6"/>
     <tableColumn id="17" xr3:uid="{705AB0EF-BD9F-4593-A5C8-9E6C4BA5D795}" name="ADV"/>
-    <tableColumn id="3" xr3:uid="{A52BA350-4626-44A2-ADDE-201A847CD93A}" name="J_AWD_Judges" dataDxfId="14"/>
+    <tableColumn id="3" xr3:uid="{A52BA350-4626-44A2-ADDE-201A847CD93A}" name="J_AWD_Judges" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5245E064-699F-4B50-AC64-10C5360A5DC3}" name="Assignments" displayName="Assignments" ref="A1:H418" totalsRowShown="0" dataDxfId="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{5245E064-699F-4B50-AC64-10C5360A5DC3}" name="Assignments" displayName="Assignments" ref="A1:H418" totalsRowShown="0" dataDxfId="61">
   <autoFilter ref="A1:H418" xr:uid="{5245E064-699F-4B50-AC64-10C5360A5DC3}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H389">
     <sortCondition ref="F1:F389"/>
   </sortState>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{C494A647-227F-40A0-AF21-8E14E63FAE7A}" name="Short Name" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{69A3FC9F-727B-4EFD-819E-768850C8CB00}" name="Team #" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{278EACB6-A801-4319-849C-E37D6EAB748F}" name="Team Name" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{8F817912-69FC-44DC-91B2-68C5C3575940}" name="Coach Name" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{4991FCB8-BE6E-4947-A78F-20515BD2B1BC}" name="Organization" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{458789FB-ACA2-4AE5-BF28-87906130022C}" name="Div" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{52B92E3D-40FD-492A-B778-6CC6A1C881B2}" name="Mem" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{78B6183D-6435-4716-A451-31227AA321DB}" name="State?" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{C494A647-227F-40A0-AF21-8E14E63FAE7A}" name="Short Name" dataDxfId="60"/>
+    <tableColumn id="2" xr3:uid="{69A3FC9F-727B-4EFD-819E-768850C8CB00}" name="Team #" dataDxfId="59"/>
+    <tableColumn id="3" xr3:uid="{278EACB6-A801-4319-849C-E37D6EAB748F}" name="Team Name" dataDxfId="58"/>
+    <tableColumn id="4" xr3:uid="{8F817912-69FC-44DC-91B2-68C5C3575940}" name="Coach Name" dataDxfId="57"/>
+    <tableColumn id="5" xr3:uid="{4991FCB8-BE6E-4947-A78F-20515BD2B1BC}" name="Organization" dataDxfId="56"/>
+    <tableColumn id="6" xr3:uid="{458789FB-ACA2-4AE5-BF28-87906130022C}" name="Div" dataDxfId="55"/>
+    <tableColumn id="7" xr3:uid="{52B92E3D-40FD-492A-B778-6CC6A1C881B2}" name="Mem" dataDxfId="54"/>
+    <tableColumn id="8" xr3:uid="{78B6183D-6435-4716-A451-31227AA321DB}" name="State?" dataDxfId="53"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -7304,7 +7304,7 @@
         <v>1</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">

</xml_diff>